<commit_message>
Marca el 12/10/2027 com a festiu al cronograma
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDkSHuGdwYQW6bQEdBsCTx
</commit_message>
<xml_diff>
--- a/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
+++ b/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
@@ -30298,7 +30298,12 @@
       <c r="AG306" s="156" t="n"/>
       <c r="AH306" s="142" t="n"/>
       <c r="AI306" s="500" t="n">
-        <v>21</v>
+        <v>20</v>
+      </c>
+      <c r="AK306" s="877" t="inlineStr">
+        <is>
+          <t>Festius: 12/10 Festa Nacional d'Espanya (Nacional)</t>
+        </is>
       </c>
     </row>
     <row r="307" ht="51" customHeight="1" s="757">
@@ -30431,7 +30436,7 @@
       <c r="L308" s="879" t="n"/>
       <c r="M308" s="879" t="n"/>
       <c r="N308" s="756" t="n"/>
-      <c r="O308" s="756" t="n"/>
+      <c r="O308" s="878" t="n"/>
       <c r="P308" s="756" t="n"/>
       <c r="Q308" s="756" t="n"/>
       <c r="R308" s="756" t="n"/>
@@ -30472,7 +30477,7 @@
       <c r="L309" s="879" t="n"/>
       <c r="M309" s="879" t="n"/>
       <c r="N309" s="756" t="n"/>
-      <c r="O309" s="756" t="n"/>
+      <c r="O309" s="878" t="n"/>
       <c r="P309" s="756" t="n"/>
       <c r="Q309" s="756" t="n"/>
       <c r="R309" s="756" t="n"/>
@@ -30513,7 +30518,7 @@
       <c r="L310" s="881" t="n"/>
       <c r="M310" s="881" t="n"/>
       <c r="N310" s="778" t="n"/>
-      <c r="O310" s="778" t="n"/>
+      <c r="O310" s="880" t="n"/>
       <c r="P310" s="778" t="n"/>
       <c r="Q310" s="778" t="n"/>
       <c r="R310" s="778" t="n"/>
@@ -30554,7 +30559,7 @@
       <c r="L311" s="879" t="n"/>
       <c r="M311" s="879" t="n"/>
       <c r="N311" s="756" t="n"/>
-      <c r="O311" s="756" t="n"/>
+      <c r="O311" s="878" t="n"/>
       <c r="P311" s="756" t="n"/>
       <c r="Q311" s="756" t="n"/>
       <c r="R311" s="756" t="n"/>
@@ -30595,7 +30600,7 @@
       <c r="L312" s="879" t="n"/>
       <c r="M312" s="879" t="n"/>
       <c r="N312" s="756" t="n"/>
-      <c r="O312" s="756" t="n"/>
+      <c r="O312" s="878" t="n"/>
       <c r="P312" s="756" t="n"/>
       <c r="Q312" s="756" t="n"/>
       <c r="R312" s="756" t="n"/>
@@ -30635,7 +30640,7 @@
       <c r="L313" s="881" t="n"/>
       <c r="M313" s="881" t="n"/>
       <c r="N313" s="778" t="n"/>
-      <c r="O313" s="778" t="n"/>
+      <c r="O313" s="880" t="n"/>
       <c r="P313" s="778" t="n"/>
       <c r="Q313" s="778" t="n"/>
       <c r="R313" s="778" t="n"/>
@@ -30675,7 +30680,7 @@
       <c r="L314" s="879" t="n"/>
       <c r="M314" s="879" t="n"/>
       <c r="N314" s="755" t="n"/>
-      <c r="O314" s="755" t="n"/>
+      <c r="O314" s="882" t="n"/>
       <c r="P314" s="756" t="n"/>
       <c r="Q314" s="756" t="n"/>
       <c r="R314" s="755" t="n"/>
@@ -30715,7 +30720,7 @@
       <c r="L315" s="879" t="n"/>
       <c r="M315" s="879" t="n"/>
       <c r="N315" s="756" t="n"/>
-      <c r="O315" s="756" t="n"/>
+      <c r="O315" s="878" t="n"/>
       <c r="P315" s="756" t="n"/>
       <c r="Q315" s="756" t="n"/>
       <c r="R315" s="756" t="n"/>
@@ -30755,7 +30760,7 @@
       <c r="L316" s="879" t="n"/>
       <c r="M316" s="879" t="n"/>
       <c r="N316" s="756" t="n"/>
-      <c r="O316" s="756" t="n"/>
+      <c r="O316" s="878" t="n"/>
       <c r="P316" s="756" t="n"/>
       <c r="Q316" s="756" t="n"/>
       <c r="R316" s="756" t="n"/>
@@ -33436,7 +33441,7 @@
     <row r="36">
       <c r="A36" s="916" t="inlineStr">
         <is>
-          <t>• Setembre-desembre 2027: festius i vacances del CALENDARI_LABORAL_2027 (els festius locals 04/09 i 15/09 hi consten com 'a omplir'; el 12/10 no hi apareix com a festiu).</t>
+          <t>• Setembre-desembre 2027: festius i vacances del CALENDARI_LABORAL_2027 (els festius locals 04/09 i 15/09 hi consten com 'a omplir'). S'hi afegeix el 12/10 com a festiu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Festius locals 04/09 i 15/09 laborables a canvi del 25/06 i 07/12
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDkSHuGdwYQW6bQEdBsCTx
</commit_message>
<xml_diff>
--- a/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
+++ b/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
@@ -1119,12 +1119,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
@@ -3597,8 +3597,8 @@
     <xf numFmtId="0" fontId="0" fillId="92" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="91" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="92" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="91" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="91" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="92" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="92" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="93" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="93" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="93" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -29775,11 +29775,11 @@
       <c r="AG293" s="156" t="n"/>
       <c r="AH293" s="142" t="n"/>
       <c r="AI293" s="500" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="AK293" s="877" t="inlineStr">
         <is>
-          <t>Festius: 04/09 Festiu local 1 (a omplir) (Local) · 11/09 Diada Nacional de Catalunya (Autonòmic) · 15/09 Festiu local 2 (a omplir) (Local)</t>
+          <t>Festius: 11/09 Diada Nacional de Catalunya (Autonòmic)</t>
         </is>
       </c>
     </row>
@@ -29904,28 +29904,28 @@
       <c r="E295" s="756" t="n"/>
       <c r="F295" s="756" t="n"/>
       <c r="G295" s="878" t="n"/>
-      <c r="H295" s="879" t="n"/>
+      <c r="H295" s="878" t="n"/>
       <c r="I295" s="756" t="n"/>
       <c r="J295" s="756" t="n"/>
       <c r="K295" s="756" t="n"/>
       <c r="L295" s="756" t="n"/>
       <c r="M295" s="756" t="n"/>
-      <c r="N295" s="878" t="n"/>
-      <c r="O295" s="879" t="n"/>
+      <c r="N295" s="879" t="n"/>
+      <c r="O295" s="878" t="n"/>
       <c r="P295" s="756" t="n"/>
       <c r="Q295" s="756" t="n"/>
-      <c r="R295" s="878" t="n"/>
+      <c r="R295" s="756" t="n"/>
       <c r="S295" s="756" t="n"/>
       <c r="T295" s="756" t="n"/>
-      <c r="U295" s="879" t="n"/>
-      <c r="V295" s="879" t="n"/>
+      <c r="U295" s="878" t="n"/>
+      <c r="V295" s="878" t="n"/>
       <c r="W295" s="756" t="n"/>
       <c r="X295" s="756" t="n"/>
       <c r="Y295" s="756" t="n"/>
       <c r="Z295" s="756" t="n"/>
       <c r="AA295" s="756" t="n"/>
-      <c r="AB295" s="879" t="n"/>
-      <c r="AC295" s="879" t="n"/>
+      <c r="AB295" s="878" t="n"/>
+      <c r="AC295" s="878" t="n"/>
       <c r="AD295" s="756" t="n"/>
       <c r="AE295" s="756" t="n"/>
       <c r="AF295" s="756" t="n"/>
@@ -29945,28 +29945,28 @@
       <c r="E296" s="756" t="n"/>
       <c r="F296" s="756" t="n"/>
       <c r="G296" s="878" t="n"/>
-      <c r="H296" s="879" t="n"/>
+      <c r="H296" s="878" t="n"/>
       <c r="I296" s="756" t="n"/>
       <c r="J296" s="756" t="n"/>
       <c r="K296" s="756" t="n"/>
       <c r="L296" s="756" t="n"/>
       <c r="M296" s="756" t="n"/>
-      <c r="N296" s="878" t="n"/>
-      <c r="O296" s="879" t="n"/>
+      <c r="N296" s="879" t="n"/>
+      <c r="O296" s="878" t="n"/>
       <c r="P296" s="756" t="n"/>
       <c r="Q296" s="756" t="n"/>
-      <c r="R296" s="878" t="n"/>
+      <c r="R296" s="756" t="n"/>
       <c r="S296" s="756" t="n"/>
       <c r="T296" s="756" t="n"/>
-      <c r="U296" s="879" t="n"/>
-      <c r="V296" s="879" t="n"/>
+      <c r="U296" s="878" t="n"/>
+      <c r="V296" s="878" t="n"/>
       <c r="W296" s="756" t="n"/>
       <c r="X296" s="756" t="n"/>
       <c r="Y296" s="756" t="n"/>
       <c r="Z296" s="756" t="n"/>
       <c r="AA296" s="756" t="n"/>
-      <c r="AB296" s="879" t="n"/>
-      <c r="AC296" s="879" t="n"/>
+      <c r="AB296" s="878" t="n"/>
+      <c r="AC296" s="878" t="n"/>
       <c r="AD296" s="756" t="n"/>
       <c r="AE296" s="756" t="n"/>
       <c r="AF296" s="756" t="n"/>
@@ -29986,28 +29986,28 @@
       <c r="E297" s="778" t="n"/>
       <c r="F297" s="778" t="n"/>
       <c r="G297" s="880" t="n"/>
-      <c r="H297" s="881" t="n"/>
+      <c r="H297" s="880" t="n"/>
       <c r="I297" s="778" t="n"/>
       <c r="J297" s="778" t="n"/>
       <c r="K297" s="778" t="n"/>
       <c r="L297" s="778" t="n"/>
       <c r="M297" s="778" t="n"/>
-      <c r="N297" s="880" t="n"/>
-      <c r="O297" s="881" t="n"/>
+      <c r="N297" s="881" t="n"/>
+      <c r="O297" s="880" t="n"/>
       <c r="P297" s="778" t="n"/>
       <c r="Q297" s="778" t="n"/>
-      <c r="R297" s="880" t="n"/>
+      <c r="R297" s="778" t="n"/>
       <c r="S297" s="778" t="n"/>
       <c r="T297" s="778" t="n"/>
-      <c r="U297" s="881" t="n"/>
-      <c r="V297" s="881" t="n"/>
+      <c r="U297" s="880" t="n"/>
+      <c r="V297" s="880" t="n"/>
       <c r="W297" s="778" t="n"/>
       <c r="X297" s="778" t="n"/>
       <c r="Y297" s="778" t="n"/>
       <c r="Z297" s="778" t="n"/>
       <c r="AA297" s="778" t="n"/>
-      <c r="AB297" s="881" t="n"/>
-      <c r="AC297" s="881" t="n"/>
+      <c r="AB297" s="880" t="n"/>
+      <c r="AC297" s="880" t="n"/>
       <c r="AD297" s="778" t="n"/>
       <c r="AE297" s="778" t="n"/>
       <c r="AF297" s="778" t="n"/>
@@ -30027,28 +30027,28 @@
       <c r="E298" s="756" t="n"/>
       <c r="F298" s="756" t="n"/>
       <c r="G298" s="878" t="n"/>
-      <c r="H298" s="879" t="n"/>
+      <c r="H298" s="878" t="n"/>
       <c r="I298" s="756" t="n"/>
       <c r="J298" s="756" t="n"/>
       <c r="K298" s="756" t="n"/>
       <c r="L298" s="756" t="n"/>
       <c r="M298" s="756" t="n"/>
-      <c r="N298" s="878" t="n"/>
-      <c r="O298" s="879" t="n"/>
+      <c r="N298" s="879" t="n"/>
+      <c r="O298" s="878" t="n"/>
       <c r="P298" s="756" t="n"/>
       <c r="Q298" s="756" t="n"/>
-      <c r="R298" s="878" t="n"/>
+      <c r="R298" s="756" t="n"/>
       <c r="S298" s="756" t="n"/>
       <c r="T298" s="756" t="n"/>
-      <c r="U298" s="879" t="n"/>
-      <c r="V298" s="879" t="n"/>
+      <c r="U298" s="878" t="n"/>
+      <c r="V298" s="878" t="n"/>
       <c r="W298" s="756" t="n"/>
       <c r="X298" s="756" t="n"/>
       <c r="Y298" s="756" t="n"/>
       <c r="Z298" s="756" t="n"/>
       <c r="AA298" s="756" t="n"/>
-      <c r="AB298" s="879" t="n"/>
-      <c r="AC298" s="879" t="n"/>
+      <c r="AB298" s="878" t="n"/>
+      <c r="AC298" s="878" t="n"/>
       <c r="AD298" s="756" t="n"/>
       <c r="AE298" s="756" t="n"/>
       <c r="AF298" s="756" t="n"/>
@@ -30068,28 +30068,28 @@
       <c r="E299" s="756" t="n"/>
       <c r="F299" s="756" t="n"/>
       <c r="G299" s="878" t="n"/>
-      <c r="H299" s="879" t="n"/>
+      <c r="H299" s="878" t="n"/>
       <c r="I299" s="756" t="n"/>
       <c r="J299" s="756" t="n"/>
       <c r="K299" s="756" t="n"/>
       <c r="L299" s="756" t="n"/>
       <c r="M299" s="756" t="n"/>
-      <c r="N299" s="878" t="n"/>
-      <c r="O299" s="879" t="n"/>
+      <c r="N299" s="879" t="n"/>
+      <c r="O299" s="878" t="n"/>
       <c r="P299" s="756" t="n"/>
       <c r="Q299" s="756" t="n"/>
-      <c r="R299" s="878" t="n"/>
+      <c r="R299" s="756" t="n"/>
       <c r="S299" s="756" t="n"/>
       <c r="T299" s="756" t="n"/>
-      <c r="U299" s="879" t="n"/>
-      <c r="V299" s="879" t="n"/>
+      <c r="U299" s="878" t="n"/>
+      <c r="V299" s="878" t="n"/>
       <c r="W299" s="756" t="n"/>
       <c r="X299" s="756" t="n"/>
       <c r="Y299" s="756" t="n"/>
       <c r="Z299" s="756" t="n"/>
       <c r="AA299" s="756" t="n"/>
-      <c r="AB299" s="879" t="n"/>
-      <c r="AC299" s="879" t="n"/>
+      <c r="AB299" s="878" t="n"/>
+      <c r="AC299" s="878" t="n"/>
       <c r="AD299" s="756" t="n"/>
       <c r="AE299" s="756" t="n"/>
       <c r="AF299" s="756" t="n"/>
@@ -30108,28 +30108,28 @@
       <c r="E300" s="778" t="n"/>
       <c r="F300" s="778" t="n"/>
       <c r="G300" s="880" t="n"/>
-      <c r="H300" s="881" t="n"/>
+      <c r="H300" s="880" t="n"/>
       <c r="I300" s="778" t="n"/>
       <c r="J300" s="778" t="n"/>
       <c r="K300" s="778" t="n"/>
       <c r="L300" s="778" t="n"/>
       <c r="M300" s="778" t="n"/>
-      <c r="N300" s="880" t="n"/>
-      <c r="O300" s="881" t="n"/>
+      <c r="N300" s="881" t="n"/>
+      <c r="O300" s="880" t="n"/>
       <c r="P300" s="778" t="n"/>
       <c r="Q300" s="778" t="n"/>
-      <c r="R300" s="880" t="n"/>
+      <c r="R300" s="778" t="n"/>
       <c r="S300" s="778" t="n"/>
       <c r="T300" s="778" t="n"/>
-      <c r="U300" s="881" t="n"/>
-      <c r="V300" s="881" t="n"/>
+      <c r="U300" s="880" t="n"/>
+      <c r="V300" s="880" t="n"/>
       <c r="W300" s="778" t="n"/>
       <c r="X300" s="778" t="n"/>
       <c r="Y300" s="778" t="n"/>
       <c r="Z300" s="778" t="n"/>
       <c r="AA300" s="778" t="n"/>
-      <c r="AB300" s="881" t="n"/>
-      <c r="AC300" s="881" t="n"/>
+      <c r="AB300" s="880" t="n"/>
+      <c r="AC300" s="880" t="n"/>
       <c r="AD300" s="778" t="n"/>
       <c r="AE300" s="778" t="n"/>
       <c r="AF300" s="778" t="n"/>
@@ -30148,28 +30148,28 @@
       <c r="E301" s="755" t="n"/>
       <c r="F301" s="756" t="n"/>
       <c r="G301" s="882" t="n"/>
-      <c r="H301" s="879" t="n"/>
+      <c r="H301" s="878" t="n"/>
       <c r="I301" s="755" t="n"/>
       <c r="J301" s="756" t="n"/>
       <c r="K301" s="755" t="n"/>
       <c r="L301" s="756" t="n"/>
       <c r="M301" s="756" t="n"/>
-      <c r="N301" s="882" t="n"/>
-      <c r="O301" s="883" t="n"/>
+      <c r="N301" s="883" t="n"/>
+      <c r="O301" s="882" t="n"/>
       <c r="P301" s="756" t="n"/>
       <c r="Q301" s="756" t="n"/>
-      <c r="R301" s="882" t="n"/>
+      <c r="R301" s="755" t="n"/>
       <c r="S301" s="756" t="n"/>
       <c r="T301" s="756" t="n"/>
-      <c r="U301" s="883" t="n"/>
-      <c r="V301" s="883" t="n"/>
+      <c r="U301" s="882" t="n"/>
+      <c r="V301" s="882" t="n"/>
       <c r="W301" s="756" t="n"/>
       <c r="X301" s="756" t="n"/>
       <c r="Y301" s="755" t="n"/>
       <c r="Z301" s="756" t="n"/>
       <c r="AA301" s="756" t="n"/>
-      <c r="AB301" s="883" t="n"/>
-      <c r="AC301" s="883" t="n"/>
+      <c r="AB301" s="882" t="n"/>
+      <c r="AC301" s="882" t="n"/>
       <c r="AD301" s="756" t="n"/>
       <c r="AE301" s="756" t="n"/>
       <c r="AF301" s="755" t="n"/>
@@ -30188,28 +30188,28 @@
       <c r="E302" s="756" t="n"/>
       <c r="F302" s="756" t="n"/>
       <c r="G302" s="878" t="n"/>
-      <c r="H302" s="879" t="n"/>
+      <c r="H302" s="878" t="n"/>
       <c r="I302" s="756" t="n"/>
       <c r="J302" s="756" t="n"/>
       <c r="K302" s="756" t="n"/>
       <c r="L302" s="756" t="n"/>
       <c r="M302" s="756" t="n"/>
-      <c r="N302" s="878" t="n"/>
-      <c r="O302" s="879" t="n"/>
+      <c r="N302" s="879" t="n"/>
+      <c r="O302" s="878" t="n"/>
       <c r="P302" s="756" t="n"/>
       <c r="Q302" s="756" t="n"/>
-      <c r="R302" s="878" t="n"/>
+      <c r="R302" s="756" t="n"/>
       <c r="S302" s="756" t="n"/>
       <c r="T302" s="756" t="n"/>
-      <c r="U302" s="879" t="n"/>
-      <c r="V302" s="879" t="n"/>
+      <c r="U302" s="878" t="n"/>
+      <c r="V302" s="878" t="n"/>
       <c r="W302" s="756" t="n"/>
       <c r="X302" s="756" t="n"/>
       <c r="Y302" s="756" t="n"/>
       <c r="Z302" s="756" t="n"/>
       <c r="AA302" s="756" t="n"/>
-      <c r="AB302" s="879" t="n"/>
-      <c r="AC302" s="879" t="n"/>
+      <c r="AB302" s="878" t="n"/>
+      <c r="AC302" s="878" t="n"/>
       <c r="AD302" s="756" t="n"/>
       <c r="AE302" s="756" t="n"/>
       <c r="AF302" s="756" t="n"/>
@@ -30228,28 +30228,28 @@
       <c r="E303" s="756" t="n"/>
       <c r="F303" s="756" t="n"/>
       <c r="G303" s="878" t="n"/>
-      <c r="H303" s="879" t="n"/>
+      <c r="H303" s="878" t="n"/>
       <c r="I303" s="756" t="n"/>
       <c r="J303" s="756" t="n"/>
       <c r="K303" s="756" t="n"/>
       <c r="L303" s="756" t="n"/>
       <c r="M303" s="756" t="n"/>
-      <c r="N303" s="878" t="n"/>
-      <c r="O303" s="879" t="n"/>
+      <c r="N303" s="879" t="n"/>
+      <c r="O303" s="878" t="n"/>
       <c r="P303" s="756" t="n"/>
       <c r="Q303" s="756" t="n"/>
-      <c r="R303" s="878" t="n"/>
+      <c r="R303" s="756" t="n"/>
       <c r="S303" s="756" t="n"/>
       <c r="T303" s="756" t="n"/>
-      <c r="U303" s="879" t="n"/>
-      <c r="V303" s="879" t="n"/>
+      <c r="U303" s="878" t="n"/>
+      <c r="V303" s="878" t="n"/>
       <c r="W303" s="756" t="n"/>
       <c r="X303" s="756" t="n"/>
       <c r="Y303" s="756" t="n"/>
       <c r="Z303" s="756" t="n"/>
       <c r="AA303" s="756" t="n"/>
-      <c r="AB303" s="879" t="n"/>
-      <c r="AC303" s="879" t="n"/>
+      <c r="AB303" s="878" t="n"/>
+      <c r="AC303" s="878" t="n"/>
       <c r="AD303" s="756" t="n"/>
       <c r="AE303" s="756" t="n"/>
       <c r="AF303" s="756" t="n"/>
@@ -30426,36 +30426,36 @@
       <c r="B308" s="11" t="n"/>
       <c r="C308" s="11" t="n"/>
       <c r="D308" s="756" t="n"/>
-      <c r="E308" s="879" t="n"/>
-      <c r="F308" s="879" t="n"/>
+      <c r="E308" s="878" t="n"/>
+      <c r="F308" s="878" t="n"/>
       <c r="G308" s="756" t="n"/>
       <c r="H308" s="756" t="n"/>
       <c r="I308" s="756" t="n"/>
       <c r="J308" s="756" t="n"/>
       <c r="K308" s="756" t="n"/>
-      <c r="L308" s="879" t="n"/>
-      <c r="M308" s="879" t="n"/>
+      <c r="L308" s="878" t="n"/>
+      <c r="M308" s="878" t="n"/>
       <c r="N308" s="756" t="n"/>
-      <c r="O308" s="878" t="n"/>
+      <c r="O308" s="879" t="n"/>
       <c r="P308" s="756" t="n"/>
       <c r="Q308" s="756" t="n"/>
       <c r="R308" s="756" t="n"/>
-      <c r="S308" s="879" t="n"/>
-      <c r="T308" s="879" t="n"/>
+      <c r="S308" s="878" t="n"/>
+      <c r="T308" s="878" t="n"/>
       <c r="U308" s="756" t="n"/>
       <c r="V308" s="756" t="n"/>
       <c r="W308" s="756" t="n"/>
       <c r="X308" s="756" t="n"/>
       <c r="Y308" s="756" t="n"/>
-      <c r="Z308" s="879" t="n"/>
-      <c r="AA308" s="879" t="n"/>
+      <c r="Z308" s="878" t="n"/>
+      <c r="AA308" s="878" t="n"/>
       <c r="AB308" s="756" t="n"/>
       <c r="AC308" s="756" t="n"/>
       <c r="AD308" s="756" t="n"/>
       <c r="AE308" s="756" t="n"/>
       <c r="AF308" s="756" t="n"/>
-      <c r="AG308" s="879" t="n"/>
-      <c r="AH308" s="879" t="n"/>
+      <c r="AG308" s="878" t="n"/>
+      <c r="AH308" s="878" t="n"/>
       <c r="AI308" s="4" t="n"/>
     </row>
     <row r="309" ht="15.75" customHeight="1" s="757">
@@ -30467,36 +30467,36 @@
       <c r="B309" s="456" t="n"/>
       <c r="C309" s="456" t="n"/>
       <c r="D309" s="782" t="n"/>
-      <c r="E309" s="879" t="n"/>
-      <c r="F309" s="879" t="n"/>
+      <c r="E309" s="878" t="n"/>
+      <c r="F309" s="878" t="n"/>
       <c r="G309" s="756" t="n"/>
       <c r="H309" s="756" t="n"/>
       <c r="I309" s="756" t="n"/>
       <c r="J309" s="756" t="n"/>
       <c r="K309" s="756" t="n"/>
-      <c r="L309" s="879" t="n"/>
-      <c r="M309" s="879" t="n"/>
+      <c r="L309" s="878" t="n"/>
+      <c r="M309" s="878" t="n"/>
       <c r="N309" s="756" t="n"/>
-      <c r="O309" s="878" t="n"/>
+      <c r="O309" s="879" t="n"/>
       <c r="P309" s="756" t="n"/>
       <c r="Q309" s="756" t="n"/>
       <c r="R309" s="756" t="n"/>
-      <c r="S309" s="879" t="n"/>
-      <c r="T309" s="879" t="n"/>
+      <c r="S309" s="878" t="n"/>
+      <c r="T309" s="878" t="n"/>
       <c r="U309" s="756" t="n"/>
       <c r="V309" s="756" t="n"/>
       <c r="W309" s="756" t="n"/>
       <c r="X309" s="756" t="n"/>
       <c r="Y309" s="756" t="n"/>
-      <c r="Z309" s="879" t="n"/>
-      <c r="AA309" s="879" t="n"/>
+      <c r="Z309" s="878" t="n"/>
+      <c r="AA309" s="878" t="n"/>
       <c r="AB309" s="756" t="n"/>
       <c r="AC309" s="756" t="n"/>
       <c r="AD309" s="756" t="n"/>
       <c r="AE309" s="756" t="n"/>
       <c r="AF309" s="756" t="n"/>
-      <c r="AG309" s="879" t="n"/>
-      <c r="AH309" s="879" t="n"/>
+      <c r="AG309" s="878" t="n"/>
+      <c r="AH309" s="878" t="n"/>
       <c r="AI309" s="4" t="n"/>
     </row>
     <row r="310" ht="19.5" customHeight="1" s="757">
@@ -30508,36 +30508,36 @@
       <c r="B310" s="15" t="n"/>
       <c r="C310" s="15" t="n"/>
       <c r="D310" s="783" t="n"/>
-      <c r="E310" s="881" t="n"/>
-      <c r="F310" s="881" t="n"/>
+      <c r="E310" s="880" t="n"/>
+      <c r="F310" s="880" t="n"/>
       <c r="G310" s="778" t="n"/>
       <c r="H310" s="778" t="n"/>
       <c r="I310" s="778" t="n"/>
       <c r="J310" s="778" t="n"/>
       <c r="K310" s="778" t="n"/>
-      <c r="L310" s="881" t="n"/>
-      <c r="M310" s="881" t="n"/>
+      <c r="L310" s="880" t="n"/>
+      <c r="M310" s="880" t="n"/>
       <c r="N310" s="778" t="n"/>
-      <c r="O310" s="880" t="n"/>
+      <c r="O310" s="881" t="n"/>
       <c r="P310" s="778" t="n"/>
       <c r="Q310" s="778" t="n"/>
       <c r="R310" s="778" t="n"/>
-      <c r="S310" s="881" t="n"/>
-      <c r="T310" s="881" t="n"/>
+      <c r="S310" s="880" t="n"/>
+      <c r="T310" s="880" t="n"/>
       <c r="U310" s="778" t="n"/>
       <c r="V310" s="778" t="n"/>
       <c r="W310" s="778" t="n"/>
       <c r="X310" s="778" t="n"/>
       <c r="Y310" s="778" t="n"/>
-      <c r="Z310" s="881" t="n"/>
-      <c r="AA310" s="881" t="n"/>
+      <c r="Z310" s="880" t="n"/>
+      <c r="AA310" s="880" t="n"/>
       <c r="AB310" s="778" t="n"/>
       <c r="AC310" s="778" t="n"/>
       <c r="AD310" s="778" t="n"/>
       <c r="AE310" s="778" t="n"/>
       <c r="AF310" s="778" t="n"/>
-      <c r="AG310" s="881" t="n"/>
-      <c r="AH310" s="881" t="n"/>
+      <c r="AG310" s="880" t="n"/>
+      <c r="AH310" s="880" t="n"/>
       <c r="AI310" s="4" t="n"/>
     </row>
     <row r="311" ht="16.5" customHeight="1" s="757">
@@ -30549,36 +30549,36 @@
       <c r="B311" s="18" t="n"/>
       <c r="C311" s="18" t="n"/>
       <c r="D311" s="755" t="n"/>
-      <c r="E311" s="879" t="n"/>
-      <c r="F311" s="879" t="n"/>
+      <c r="E311" s="878" t="n"/>
+      <c r="F311" s="878" t="n"/>
       <c r="G311" s="756" t="n"/>
       <c r="H311" s="756" t="n"/>
       <c r="I311" s="756" t="n"/>
       <c r="J311" s="756" t="n"/>
       <c r="K311" s="756" t="n"/>
-      <c r="L311" s="879" t="n"/>
-      <c r="M311" s="879" t="n"/>
+      <c r="L311" s="878" t="n"/>
+      <c r="M311" s="878" t="n"/>
       <c r="N311" s="756" t="n"/>
-      <c r="O311" s="878" t="n"/>
+      <c r="O311" s="879" t="n"/>
       <c r="P311" s="756" t="n"/>
       <c r="Q311" s="756" t="n"/>
       <c r="R311" s="756" t="n"/>
-      <c r="S311" s="879" t="n"/>
-      <c r="T311" s="879" t="n"/>
+      <c r="S311" s="878" t="n"/>
+      <c r="T311" s="878" t="n"/>
       <c r="U311" s="756" t="n"/>
       <c r="V311" s="756" t="n"/>
       <c r="W311" s="756" t="n"/>
       <c r="X311" s="756" t="n"/>
       <c r="Y311" s="756" t="n"/>
-      <c r="Z311" s="879" t="n"/>
-      <c r="AA311" s="879" t="n"/>
+      <c r="Z311" s="878" t="n"/>
+      <c r="AA311" s="878" t="n"/>
       <c r="AB311" s="756" t="n"/>
       <c r="AC311" s="756" t="n"/>
       <c r="AD311" s="756" t="n"/>
       <c r="AE311" s="756" t="n"/>
       <c r="AF311" s="756" t="n"/>
-      <c r="AG311" s="879" t="n"/>
-      <c r="AH311" s="879" t="n"/>
+      <c r="AG311" s="878" t="n"/>
+      <c r="AH311" s="878" t="n"/>
       <c r="AI311" s="4" t="n"/>
     </row>
     <row r="312" ht="15.75" customHeight="1" s="757">
@@ -30590,36 +30590,36 @@
       <c r="B312" s="11" t="n"/>
       <c r="C312" s="11" t="n"/>
       <c r="D312" s="756" t="n"/>
-      <c r="E312" s="879" t="n"/>
-      <c r="F312" s="879" t="n"/>
+      <c r="E312" s="878" t="n"/>
+      <c r="F312" s="878" t="n"/>
       <c r="G312" s="756" t="n"/>
       <c r="H312" s="756" t="n"/>
       <c r="I312" s="756" t="n"/>
       <c r="J312" s="756" t="n"/>
       <c r="K312" s="756" t="n"/>
-      <c r="L312" s="879" t="n"/>
-      <c r="M312" s="879" t="n"/>
+      <c r="L312" s="878" t="n"/>
+      <c r="M312" s="878" t="n"/>
       <c r="N312" s="756" t="n"/>
-      <c r="O312" s="878" t="n"/>
+      <c r="O312" s="879" t="n"/>
       <c r="P312" s="756" t="n"/>
       <c r="Q312" s="756" t="n"/>
       <c r="R312" s="756" t="n"/>
-      <c r="S312" s="879" t="n"/>
-      <c r="T312" s="879" t="n"/>
+      <c r="S312" s="878" t="n"/>
+      <c r="T312" s="878" t="n"/>
       <c r="U312" s="756" t="n"/>
       <c r="V312" s="756" t="n"/>
       <c r="W312" s="756" t="n"/>
       <c r="X312" s="756" t="n"/>
       <c r="Y312" s="756" t="n"/>
-      <c r="Z312" s="879" t="n"/>
-      <c r="AA312" s="879" t="n"/>
+      <c r="Z312" s="878" t="n"/>
+      <c r="AA312" s="878" t="n"/>
       <c r="AB312" s="756" t="n"/>
       <c r="AC312" s="756" t="n"/>
       <c r="AD312" s="756" t="n"/>
       <c r="AE312" s="756" t="n"/>
       <c r="AF312" s="756" t="n"/>
-      <c r="AG312" s="879" t="n"/>
-      <c r="AH312" s="879" t="n"/>
+      <c r="AG312" s="878" t="n"/>
+      <c r="AH312" s="878" t="n"/>
     </row>
     <row r="313" ht="16.5" customHeight="1" s="757">
       <c r="A313" s="14" t="inlineStr">
@@ -30630,36 +30630,36 @@
       <c r="B313" s="15" t="n"/>
       <c r="C313" s="15" t="n"/>
       <c r="D313" s="783" t="n"/>
-      <c r="E313" s="881" t="n"/>
-      <c r="F313" s="881" t="n"/>
+      <c r="E313" s="880" t="n"/>
+      <c r="F313" s="880" t="n"/>
       <c r="G313" s="778" t="n"/>
       <c r="H313" s="778" t="n"/>
       <c r="I313" s="778" t="n"/>
       <c r="J313" s="778" t="n"/>
       <c r="K313" s="778" t="n"/>
-      <c r="L313" s="881" t="n"/>
-      <c r="M313" s="881" t="n"/>
+      <c r="L313" s="880" t="n"/>
+      <c r="M313" s="880" t="n"/>
       <c r="N313" s="778" t="n"/>
-      <c r="O313" s="880" t="n"/>
+      <c r="O313" s="881" t="n"/>
       <c r="P313" s="778" t="n"/>
       <c r="Q313" s="778" t="n"/>
       <c r="R313" s="778" t="n"/>
-      <c r="S313" s="881" t="n"/>
-      <c r="T313" s="881" t="n"/>
+      <c r="S313" s="880" t="n"/>
+      <c r="T313" s="880" t="n"/>
       <c r="U313" s="778" t="n"/>
       <c r="V313" s="778" t="n"/>
       <c r="W313" s="778" t="n"/>
       <c r="X313" s="778" t="n"/>
       <c r="Y313" s="778" t="n"/>
-      <c r="Z313" s="881" t="n"/>
-      <c r="AA313" s="881" t="n"/>
+      <c r="Z313" s="880" t="n"/>
+      <c r="AA313" s="880" t="n"/>
       <c r="AB313" s="778" t="n"/>
       <c r="AC313" s="778" t="n"/>
       <c r="AD313" s="778" t="n"/>
       <c r="AE313" s="778" t="n"/>
       <c r="AF313" s="778" t="n"/>
-      <c r="AG313" s="881" t="n"/>
-      <c r="AH313" s="881" t="n"/>
+      <c r="AG313" s="880" t="n"/>
+      <c r="AH313" s="880" t="n"/>
     </row>
     <row r="314" ht="16.5" customHeight="1" s="757">
       <c r="A314" s="10" t="inlineStr">
@@ -30670,36 +30670,36 @@
       <c r="B314" s="11" t="n"/>
       <c r="C314" s="11" t="n"/>
       <c r="D314" s="755" t="n"/>
-      <c r="E314" s="883" t="n"/>
-      <c r="F314" s="879" t="n"/>
+      <c r="E314" s="882" t="n"/>
+      <c r="F314" s="878" t="n"/>
       <c r="G314" s="755" t="n"/>
       <c r="H314" s="756" t="n"/>
       <c r="I314" s="755" t="n"/>
       <c r="J314" s="756" t="n"/>
       <c r="K314" s="755" t="n"/>
-      <c r="L314" s="879" t="n"/>
-      <c r="M314" s="879" t="n"/>
+      <c r="L314" s="878" t="n"/>
+      <c r="M314" s="878" t="n"/>
       <c r="N314" s="755" t="n"/>
-      <c r="O314" s="882" t="n"/>
+      <c r="O314" s="883" t="n"/>
       <c r="P314" s="756" t="n"/>
       <c r="Q314" s="756" t="n"/>
       <c r="R314" s="755" t="n"/>
-      <c r="S314" s="879" t="n"/>
-      <c r="T314" s="879" t="n"/>
+      <c r="S314" s="878" t="n"/>
+      <c r="T314" s="878" t="n"/>
       <c r="U314" s="755" t="n"/>
       <c r="V314" s="755" t="n"/>
       <c r="W314" s="756" t="n"/>
       <c r="X314" s="756" t="n"/>
       <c r="Y314" s="755" t="n"/>
-      <c r="Z314" s="879" t="n"/>
-      <c r="AA314" s="879" t="n"/>
+      <c r="Z314" s="878" t="n"/>
+      <c r="AA314" s="878" t="n"/>
       <c r="AB314" s="755" t="n"/>
       <c r="AC314" s="755" t="n"/>
       <c r="AD314" s="756" t="n"/>
       <c r="AE314" s="756" t="n"/>
       <c r="AF314" s="755" t="n"/>
-      <c r="AG314" s="879" t="n"/>
-      <c r="AH314" s="879" t="n"/>
+      <c r="AG314" s="878" t="n"/>
+      <c r="AH314" s="878" t="n"/>
     </row>
     <row r="315" ht="15.75" customHeight="1" s="757">
       <c r="A315" s="12" t="inlineStr">
@@ -30710,36 +30710,36 @@
       <c r="B315" s="11" t="n"/>
       <c r="C315" s="11" t="n"/>
       <c r="D315" s="756" t="n"/>
-      <c r="E315" s="879" t="n"/>
-      <c r="F315" s="879" t="n"/>
+      <c r="E315" s="878" t="n"/>
+      <c r="F315" s="878" t="n"/>
       <c r="G315" s="756" t="n"/>
       <c r="H315" s="756" t="n"/>
       <c r="I315" s="756" t="n"/>
       <c r="J315" s="756" t="n"/>
       <c r="K315" s="756" t="n"/>
-      <c r="L315" s="879" t="n"/>
-      <c r="M315" s="879" t="n"/>
+      <c r="L315" s="878" t="n"/>
+      <c r="M315" s="878" t="n"/>
       <c r="N315" s="756" t="n"/>
-      <c r="O315" s="878" t="n"/>
+      <c r="O315" s="879" t="n"/>
       <c r="P315" s="756" t="n"/>
       <c r="Q315" s="756" t="n"/>
       <c r="R315" s="756" t="n"/>
-      <c r="S315" s="879" t="n"/>
-      <c r="T315" s="879" t="n"/>
+      <c r="S315" s="878" t="n"/>
+      <c r="T315" s="878" t="n"/>
       <c r="U315" s="756" t="n"/>
       <c r="V315" s="756" t="n"/>
       <c r="W315" s="756" t="n"/>
       <c r="X315" s="756" t="n"/>
       <c r="Y315" s="756" t="n"/>
-      <c r="Z315" s="879" t="n"/>
-      <c r="AA315" s="879" t="n"/>
+      <c r="Z315" s="878" t="n"/>
+      <c r="AA315" s="878" t="n"/>
       <c r="AB315" s="756" t="n"/>
       <c r="AC315" s="756" t="n"/>
       <c r="AD315" s="756" t="n"/>
       <c r="AE315" s="756" t="n"/>
       <c r="AF315" s="756" t="n"/>
-      <c r="AG315" s="879" t="n"/>
-      <c r="AH315" s="879" t="n"/>
+      <c r="AG315" s="878" t="n"/>
+      <c r="AH315" s="878" t="n"/>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="757">
       <c r="A316" s="12" t="inlineStr">
@@ -30750,36 +30750,36 @@
       <c r="B316" s="11" t="n"/>
       <c r="C316" s="11" t="n"/>
       <c r="D316" s="756" t="n"/>
-      <c r="E316" s="879" t="n"/>
-      <c r="F316" s="879" t="n"/>
+      <c r="E316" s="878" t="n"/>
+      <c r="F316" s="878" t="n"/>
       <c r="G316" s="756" t="n"/>
       <c r="H316" s="756" t="n"/>
       <c r="I316" s="756" t="n"/>
       <c r="J316" s="756" t="n"/>
       <c r="K316" s="756" t="n"/>
-      <c r="L316" s="879" t="n"/>
-      <c r="M316" s="879" t="n"/>
+      <c r="L316" s="878" t="n"/>
+      <c r="M316" s="878" t="n"/>
       <c r="N316" s="756" t="n"/>
-      <c r="O316" s="878" t="n"/>
+      <c r="O316" s="879" t="n"/>
       <c r="P316" s="756" t="n"/>
       <c r="Q316" s="756" t="n"/>
       <c r="R316" s="756" t="n"/>
-      <c r="S316" s="879" t="n"/>
-      <c r="T316" s="879" t="n"/>
+      <c r="S316" s="878" t="n"/>
+      <c r="T316" s="878" t="n"/>
       <c r="U316" s="756" t="n"/>
       <c r="V316" s="756" t="n"/>
       <c r="W316" s="756" t="n"/>
       <c r="X316" s="756" t="n"/>
       <c r="Y316" s="756" t="n"/>
-      <c r="Z316" s="879" t="n"/>
-      <c r="AA316" s="879" t="n"/>
+      <c r="Z316" s="878" t="n"/>
+      <c r="AA316" s="878" t="n"/>
       <c r="AB316" s="756" t="n"/>
       <c r="AC316" s="756" t="n"/>
       <c r="AD316" s="756" t="n"/>
       <c r="AE316" s="756" t="n"/>
       <c r="AF316" s="756" t="n"/>
-      <c r="AG316" s="879" t="n"/>
-      <c r="AH316" s="879" t="n"/>
+      <c r="AG316" s="878" t="n"/>
+      <c r="AH316" s="878" t="n"/>
     </row>
     <row r="317" s="757"/>
     <row r="318" s="757"/>
@@ -30948,34 +30948,34 @@
       </c>
       <c r="B321" s="11" t="n"/>
       <c r="C321" s="11" t="n"/>
-      <c r="D321" s="878" t="n"/>
+      <c r="D321" s="879" t="n"/>
       <c r="E321" s="756" t="n"/>
       <c r="F321" s="756" t="n"/>
       <c r="G321" s="756" t="n"/>
       <c r="H321" s="756" t="n"/>
-      <c r="I321" s="879" t="n"/>
-      <c r="J321" s="879" t="n"/>
+      <c r="I321" s="878" t="n"/>
+      <c r="J321" s="878" t="n"/>
       <c r="K321" s="756" t="n"/>
       <c r="L321" s="756" t="n"/>
       <c r="M321" s="756" t="n"/>
       <c r="N321" s="756" t="n"/>
       <c r="O321" s="756" t="n"/>
-      <c r="P321" s="879" t="n"/>
-      <c r="Q321" s="879" t="n"/>
+      <c r="P321" s="878" t="n"/>
+      <c r="Q321" s="878" t="n"/>
       <c r="R321" s="756" t="n"/>
       <c r="S321" s="756" t="n"/>
       <c r="T321" s="756" t="n"/>
       <c r="U321" s="756" t="n"/>
       <c r="V321" s="756" t="n"/>
-      <c r="W321" s="879" t="n"/>
-      <c r="X321" s="879" t="n"/>
+      <c r="W321" s="878" t="n"/>
+      <c r="X321" s="878" t="n"/>
       <c r="Y321" s="756" t="n"/>
       <c r="Z321" s="756" t="n"/>
       <c r="AA321" s="756" t="n"/>
       <c r="AB321" s="756" t="n"/>
       <c r="AC321" s="756" t="n"/>
-      <c r="AD321" s="879" t="n"/>
-      <c r="AE321" s="879" t="n"/>
+      <c r="AD321" s="878" t="n"/>
+      <c r="AE321" s="878" t="n"/>
       <c r="AF321" s="756" t="n"/>
       <c r="AG321" s="756" t="n"/>
       <c r="AH321" s="756" t="n"/>
@@ -30994,29 +30994,29 @@
       <c r="F322" s="756" t="n"/>
       <c r="G322" s="756" t="n"/>
       <c r="H322" s="756" t="n"/>
-      <c r="I322" s="879" t="n"/>
-      <c r="J322" s="879" t="n"/>
+      <c r="I322" s="878" t="n"/>
+      <c r="J322" s="878" t="n"/>
       <c r="K322" s="756" t="n"/>
       <c r="L322" s="756" t="n"/>
       <c r="M322" s="756" t="n"/>
       <c r="N322" s="756" t="n"/>
       <c r="O322" s="756" t="n"/>
-      <c r="P322" s="879" t="n"/>
-      <c r="Q322" s="879" t="n"/>
+      <c r="P322" s="878" t="n"/>
+      <c r="Q322" s="878" t="n"/>
       <c r="R322" s="756" t="n"/>
       <c r="S322" s="756" t="n"/>
       <c r="T322" s="756" t="n"/>
       <c r="U322" s="756" t="n"/>
       <c r="V322" s="756" t="n"/>
-      <c r="W322" s="879" t="n"/>
-      <c r="X322" s="879" t="n"/>
+      <c r="W322" s="878" t="n"/>
+      <c r="X322" s="878" t="n"/>
       <c r="Y322" s="756" t="n"/>
       <c r="Z322" s="756" t="n"/>
       <c r="AA322" s="756" t="n"/>
       <c r="AB322" s="756" t="n"/>
       <c r="AC322" s="756" t="n"/>
-      <c r="AD322" s="879" t="n"/>
-      <c r="AE322" s="879" t="n"/>
+      <c r="AD322" s="878" t="n"/>
+      <c r="AE322" s="878" t="n"/>
       <c r="AF322" s="756" t="n"/>
       <c r="AG322" s="756" t="n"/>
       <c r="AH322" s="756" t="n"/>
@@ -31035,29 +31035,29 @@
       <c r="F323" s="778" t="n"/>
       <c r="G323" s="778" t="n"/>
       <c r="H323" s="778" t="n"/>
-      <c r="I323" s="881" t="n"/>
-      <c r="J323" s="881" t="n"/>
+      <c r="I323" s="880" t="n"/>
+      <c r="J323" s="880" t="n"/>
       <c r="K323" s="778" t="n"/>
       <c r="L323" s="778" t="n"/>
       <c r="M323" s="778" t="n"/>
       <c r="N323" s="778" t="n"/>
       <c r="O323" s="778" t="n"/>
-      <c r="P323" s="881" t="n"/>
-      <c r="Q323" s="881" t="n"/>
+      <c r="P323" s="880" t="n"/>
+      <c r="Q323" s="880" t="n"/>
       <c r="R323" s="778" t="n"/>
       <c r="S323" s="778" t="n"/>
       <c r="T323" s="778" t="n"/>
       <c r="U323" s="778" t="n"/>
       <c r="V323" s="778" t="n"/>
-      <c r="W323" s="881" t="n"/>
-      <c r="X323" s="881" t="n"/>
+      <c r="W323" s="880" t="n"/>
+      <c r="X323" s="880" t="n"/>
       <c r="Y323" s="778" t="n"/>
       <c r="Z323" s="778" t="n"/>
       <c r="AA323" s="778" t="n"/>
       <c r="AB323" s="778" t="n"/>
       <c r="AC323" s="778" t="n"/>
-      <c r="AD323" s="881" t="n"/>
-      <c r="AE323" s="881" t="n"/>
+      <c r="AD323" s="880" t="n"/>
+      <c r="AE323" s="880" t="n"/>
       <c r="AF323" s="778" t="n"/>
       <c r="AG323" s="778" t="n"/>
       <c r="AH323" s="778" t="n"/>
@@ -31071,34 +31071,34 @@
       </c>
       <c r="B324" s="18" t="n"/>
       <c r="C324" s="18" t="n"/>
-      <c r="D324" s="882" t="n"/>
+      <c r="D324" s="883" t="n"/>
       <c r="E324" s="756" t="n"/>
       <c r="F324" s="756" t="n"/>
       <c r="G324" s="756" t="n"/>
       <c r="H324" s="756" t="n"/>
-      <c r="I324" s="879" t="n"/>
-      <c r="J324" s="879" t="n"/>
+      <c r="I324" s="878" t="n"/>
+      <c r="J324" s="878" t="n"/>
       <c r="K324" s="756" t="n"/>
       <c r="L324" s="756" t="n"/>
       <c r="M324" s="756" t="n"/>
       <c r="N324" s="756" t="n"/>
       <c r="O324" s="756" t="n"/>
-      <c r="P324" s="879" t="n"/>
-      <c r="Q324" s="879" t="n"/>
+      <c r="P324" s="878" t="n"/>
+      <c r="Q324" s="878" t="n"/>
       <c r="R324" s="756" t="n"/>
       <c r="S324" s="756" t="n"/>
       <c r="T324" s="756" t="n"/>
       <c r="U324" s="756" t="n"/>
       <c r="V324" s="756" t="n"/>
-      <c r="W324" s="879" t="n"/>
-      <c r="X324" s="879" t="n"/>
+      <c r="W324" s="878" t="n"/>
+      <c r="X324" s="878" t="n"/>
       <c r="Y324" s="756" t="n"/>
       <c r="Z324" s="756" t="n"/>
       <c r="AA324" s="756" t="n"/>
       <c r="AB324" s="756" t="n"/>
       <c r="AC324" s="756" t="n"/>
-      <c r="AD324" s="879" t="n"/>
-      <c r="AE324" s="879" t="n"/>
+      <c r="AD324" s="878" t="n"/>
+      <c r="AE324" s="878" t="n"/>
       <c r="AF324" s="756" t="n"/>
       <c r="AG324" s="756" t="n"/>
       <c r="AH324" s="756" t="n"/>
@@ -31112,34 +31112,34 @@
       </c>
       <c r="B325" s="11" t="n"/>
       <c r="C325" s="11" t="n"/>
-      <c r="D325" s="878" t="n"/>
+      <c r="D325" s="879" t="n"/>
       <c r="E325" s="756" t="n"/>
       <c r="F325" s="756" t="n"/>
       <c r="G325" s="756" t="n"/>
       <c r="H325" s="756" t="n"/>
-      <c r="I325" s="879" t="n"/>
-      <c r="J325" s="879" t="n"/>
+      <c r="I325" s="878" t="n"/>
+      <c r="J325" s="878" t="n"/>
       <c r="K325" s="756" t="n"/>
       <c r="L325" s="756" t="n"/>
       <c r="M325" s="756" t="n"/>
       <c r="N325" s="756" t="n"/>
       <c r="O325" s="756" t="n"/>
-      <c r="P325" s="879" t="n"/>
-      <c r="Q325" s="879" t="n"/>
+      <c r="P325" s="878" t="n"/>
+      <c r="Q325" s="878" t="n"/>
       <c r="R325" s="756" t="n"/>
       <c r="S325" s="756" t="n"/>
       <c r="T325" s="756" t="n"/>
       <c r="U325" s="756" t="n"/>
       <c r="V325" s="756" t="n"/>
-      <c r="W325" s="879" t="n"/>
-      <c r="X325" s="879" t="n"/>
+      <c r="W325" s="878" t="n"/>
+      <c r="X325" s="878" t="n"/>
       <c r="Y325" s="756" t="n"/>
       <c r="Z325" s="756" t="n"/>
       <c r="AA325" s="756" t="n"/>
       <c r="AB325" s="756" t="n"/>
       <c r="AC325" s="756" t="n"/>
-      <c r="AD325" s="879" t="n"/>
-      <c r="AE325" s="879" t="n"/>
+      <c r="AD325" s="878" t="n"/>
+      <c r="AE325" s="878" t="n"/>
       <c r="AF325" s="756" t="n"/>
       <c r="AG325" s="756" t="n"/>
       <c r="AH325" s="756" t="n"/>
@@ -31157,29 +31157,29 @@
       <c r="F326" s="778" t="n"/>
       <c r="G326" s="778" t="n"/>
       <c r="H326" s="778" t="n"/>
-      <c r="I326" s="881" t="n"/>
-      <c r="J326" s="881" t="n"/>
+      <c r="I326" s="880" t="n"/>
+      <c r="J326" s="880" t="n"/>
       <c r="K326" s="778" t="n"/>
       <c r="L326" s="778" t="n"/>
       <c r="M326" s="778" t="n"/>
       <c r="N326" s="778" t="n"/>
       <c r="O326" s="778" t="n"/>
-      <c r="P326" s="881" t="n"/>
-      <c r="Q326" s="881" t="n"/>
+      <c r="P326" s="880" t="n"/>
+      <c r="Q326" s="880" t="n"/>
       <c r="R326" s="778" t="n"/>
       <c r="S326" s="778" t="n"/>
       <c r="T326" s="778" t="n"/>
       <c r="U326" s="778" t="n"/>
       <c r="V326" s="778" t="n"/>
-      <c r="W326" s="881" t="n"/>
-      <c r="X326" s="881" t="n"/>
+      <c r="W326" s="880" t="n"/>
+      <c r="X326" s="880" t="n"/>
       <c r="Y326" s="778" t="n"/>
       <c r="Z326" s="778" t="n"/>
       <c r="AA326" s="778" t="n"/>
       <c r="AB326" s="778" t="n"/>
       <c r="AC326" s="778" t="n"/>
-      <c r="AD326" s="881" t="n"/>
-      <c r="AE326" s="881" t="n"/>
+      <c r="AD326" s="880" t="n"/>
+      <c r="AE326" s="880" t="n"/>
       <c r="AF326" s="778" t="n"/>
       <c r="AG326" s="778" t="n"/>
       <c r="AH326" s="778" t="n"/>
@@ -31192,34 +31192,34 @@
       </c>
       <c r="B327" s="11" t="n"/>
       <c r="C327" s="11" t="n"/>
-      <c r="D327" s="882" t="n"/>
+      <c r="D327" s="883" t="n"/>
       <c r="E327" s="755" t="n"/>
       <c r="F327" s="756" t="n"/>
       <c r="G327" s="755" t="n"/>
       <c r="H327" s="756" t="n"/>
-      <c r="I327" s="883" t="n"/>
-      <c r="J327" s="879" t="n"/>
+      <c r="I327" s="882" t="n"/>
+      <c r="J327" s="878" t="n"/>
       <c r="K327" s="755" t="n"/>
       <c r="L327" s="756" t="n"/>
       <c r="M327" s="756" t="n"/>
       <c r="N327" s="755" t="n"/>
       <c r="O327" s="755" t="n"/>
-      <c r="P327" s="879" t="n"/>
-      <c r="Q327" s="879" t="n"/>
+      <c r="P327" s="878" t="n"/>
+      <c r="Q327" s="878" t="n"/>
       <c r="R327" s="755" t="n"/>
       <c r="S327" s="756" t="n"/>
       <c r="T327" s="756" t="n"/>
       <c r="U327" s="755" t="n"/>
       <c r="V327" s="755" t="n"/>
-      <c r="W327" s="879" t="n"/>
-      <c r="X327" s="879" t="n"/>
+      <c r="W327" s="878" t="n"/>
+      <c r="X327" s="878" t="n"/>
       <c r="Y327" s="755" t="n"/>
       <c r="Z327" s="756" t="n"/>
       <c r="AA327" s="756" t="n"/>
       <c r="AB327" s="755" t="n"/>
       <c r="AC327" s="755" t="n"/>
-      <c r="AD327" s="879" t="n"/>
-      <c r="AE327" s="879" t="n"/>
+      <c r="AD327" s="878" t="n"/>
+      <c r="AE327" s="878" t="n"/>
       <c r="AF327" s="755" t="n"/>
       <c r="AG327" s="756" t="n"/>
       <c r="AH327" s="756" t="n"/>
@@ -31232,34 +31232,34 @@
       </c>
       <c r="B328" s="11" t="n"/>
       <c r="C328" s="11" t="n"/>
-      <c r="D328" s="878" t="n"/>
+      <c r="D328" s="879" t="n"/>
       <c r="E328" s="756" t="n"/>
       <c r="F328" s="756" t="n"/>
       <c r="G328" s="756" t="n"/>
       <c r="H328" s="756" t="n"/>
-      <c r="I328" s="879" t="n"/>
-      <c r="J328" s="879" t="n"/>
+      <c r="I328" s="878" t="n"/>
+      <c r="J328" s="878" t="n"/>
       <c r="K328" s="756" t="n"/>
       <c r="L328" s="756" t="n"/>
       <c r="M328" s="756" t="n"/>
       <c r="N328" s="756" t="n"/>
       <c r="O328" s="756" t="n"/>
-      <c r="P328" s="879" t="n"/>
-      <c r="Q328" s="879" t="n"/>
+      <c r="P328" s="878" t="n"/>
+      <c r="Q328" s="878" t="n"/>
       <c r="R328" s="756" t="n"/>
       <c r="S328" s="756" t="n"/>
       <c r="T328" s="756" t="n"/>
       <c r="U328" s="756" t="n"/>
       <c r="V328" s="756" t="n"/>
-      <c r="W328" s="879" t="n"/>
-      <c r="X328" s="879" t="n"/>
+      <c r="W328" s="878" t="n"/>
+      <c r="X328" s="878" t="n"/>
       <c r="Y328" s="756" t="n"/>
       <c r="Z328" s="756" t="n"/>
       <c r="AA328" s="756" t="n"/>
       <c r="AB328" s="756" t="n"/>
       <c r="AC328" s="756" t="n"/>
-      <c r="AD328" s="879" t="n"/>
-      <c r="AE328" s="879" t="n"/>
+      <c r="AD328" s="878" t="n"/>
+      <c r="AE328" s="878" t="n"/>
       <c r="AF328" s="756" t="n"/>
       <c r="AG328" s="756" t="n"/>
       <c r="AH328" s="756" t="n"/>
@@ -31272,34 +31272,34 @@
       </c>
       <c r="B329" s="11" t="n"/>
       <c r="C329" s="11" t="n"/>
-      <c r="D329" s="878" t="n"/>
+      <c r="D329" s="879" t="n"/>
       <c r="E329" s="756" t="n"/>
       <c r="F329" s="756" t="n"/>
       <c r="G329" s="756" t="n"/>
       <c r="H329" s="756" t="n"/>
-      <c r="I329" s="879" t="n"/>
-      <c r="J329" s="879" t="n"/>
+      <c r="I329" s="878" t="n"/>
+      <c r="J329" s="878" t="n"/>
       <c r="K329" s="756" t="n"/>
       <c r="L329" s="756" t="n"/>
       <c r="M329" s="756" t="n"/>
       <c r="N329" s="756" t="n"/>
       <c r="O329" s="756" t="n"/>
-      <c r="P329" s="879" t="n"/>
-      <c r="Q329" s="879" t="n"/>
+      <c r="P329" s="878" t="n"/>
+      <c r="Q329" s="878" t="n"/>
       <c r="R329" s="756" t="n"/>
       <c r="S329" s="756" t="n"/>
       <c r="T329" s="756" t="n"/>
       <c r="U329" s="756" t="n"/>
       <c r="V329" s="756" t="n"/>
-      <c r="W329" s="879" t="n"/>
-      <c r="X329" s="879" t="n"/>
+      <c r="W329" s="878" t="n"/>
+      <c r="X329" s="878" t="n"/>
       <c r="Y329" s="756" t="n"/>
       <c r="Z329" s="756" t="n"/>
       <c r="AA329" s="756" t="n"/>
       <c r="AB329" s="756" t="n"/>
       <c r="AC329" s="756" t="n"/>
-      <c r="AD329" s="879" t="n"/>
-      <c r="AE329" s="879" t="n"/>
+      <c r="AD329" s="878" t="n"/>
+      <c r="AE329" s="878" t="n"/>
       <c r="AF329" s="756" t="n"/>
       <c r="AG329" s="756" t="n"/>
       <c r="AH329" s="756" t="n"/>
@@ -31346,11 +31346,11 @@
       <c r="AG332" s="156" t="n"/>
       <c r="AH332" s="142" t="n"/>
       <c r="AI332" s="500" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AK332" s="877" t="inlineStr">
         <is>
-          <t>Festius: 06/12 Dia de la Constitució (Nacional) · 08/12 Immaculada Concepció (Nacional) · 25/12 Nadal (Nacional) · Vacances: 23/12–31/12</t>
+          <t>Festius: 06/12 Dia de la Constitució (Nacional) · 07/12 Festiu local (canvi pel 15/09) · 08/12 Immaculada Concepció (Nacional) · 25/12 Nadal (Nacional) · Vacances: 23/12–31/12</t>
         </is>
       </c>
     </row>
@@ -31476,29 +31476,29 @@
       <c r="D334" s="756" t="n"/>
       <c r="E334" s="756" t="n"/>
       <c r="F334" s="756" t="n"/>
-      <c r="G334" s="879" t="n"/>
-      <c r="H334" s="879" t="n"/>
-      <c r="I334" s="878" t="n"/>
-      <c r="J334" s="756" t="n"/>
-      <c r="K334" s="878" t="n"/>
+      <c r="G334" s="878" t="n"/>
+      <c r="H334" s="878" t="n"/>
+      <c r="I334" s="879" t="n"/>
+      <c r="J334" s="879" t="n"/>
+      <c r="K334" s="879" t="n"/>
       <c r="L334" s="756" t="n"/>
       <c r="M334" s="756" t="n"/>
-      <c r="N334" s="879" t="n"/>
-      <c r="O334" s="879" t="n"/>
+      <c r="N334" s="878" t="n"/>
+      <c r="O334" s="878" t="n"/>
       <c r="P334" s="756" t="n"/>
       <c r="Q334" s="756" t="n"/>
       <c r="R334" s="756" t="n"/>
       <c r="S334" s="756" t="n"/>
       <c r="T334" s="756" t="n"/>
-      <c r="U334" s="879" t="n"/>
-      <c r="V334" s="879" t="n"/>
+      <c r="U334" s="878" t="n"/>
+      <c r="V334" s="878" t="n"/>
       <c r="W334" s="756" t="n"/>
       <c r="X334" s="756" t="n"/>
       <c r="Y334" s="756" t="n"/>
       <c r="Z334" s="886" t="n"/>
       <c r="AA334" s="886" t="n"/>
-      <c r="AB334" s="878" t="n"/>
-      <c r="AC334" s="879" t="n"/>
+      <c r="AB334" s="879" t="n"/>
+      <c r="AC334" s="878" t="n"/>
       <c r="AD334" s="886" t="n"/>
       <c r="AE334" s="886" t="n"/>
       <c r="AF334" s="886" t="n"/>
@@ -31517,29 +31517,29 @@
       <c r="D335" s="782" t="n"/>
       <c r="E335" s="756" t="n"/>
       <c r="F335" s="756" t="n"/>
-      <c r="G335" s="879" t="n"/>
-      <c r="H335" s="879" t="n"/>
-      <c r="I335" s="878" t="n"/>
-      <c r="J335" s="756" t="n"/>
-      <c r="K335" s="878" t="n"/>
+      <c r="G335" s="878" t="n"/>
+      <c r="H335" s="878" t="n"/>
+      <c r="I335" s="879" t="n"/>
+      <c r="J335" s="879" t="n"/>
+      <c r="K335" s="879" t="n"/>
       <c r="L335" s="756" t="n"/>
       <c r="M335" s="756" t="n"/>
-      <c r="N335" s="879" t="n"/>
-      <c r="O335" s="879" t="n"/>
+      <c r="N335" s="878" t="n"/>
+      <c r="O335" s="878" t="n"/>
       <c r="P335" s="756" t="n"/>
       <c r="Q335" s="756" t="n"/>
       <c r="R335" s="756" t="n"/>
       <c r="S335" s="756" t="n"/>
       <c r="T335" s="756" t="n"/>
-      <c r="U335" s="879" t="n"/>
-      <c r="V335" s="879" t="n"/>
+      <c r="U335" s="878" t="n"/>
+      <c r="V335" s="878" t="n"/>
       <c r="W335" s="756" t="n"/>
       <c r="X335" s="756" t="n"/>
       <c r="Y335" s="756" t="n"/>
       <c r="Z335" s="886" t="n"/>
       <c r="AA335" s="886" t="n"/>
-      <c r="AB335" s="878" t="n"/>
-      <c r="AC335" s="879" t="n"/>
+      <c r="AB335" s="879" t="n"/>
+      <c r="AC335" s="878" t="n"/>
       <c r="AD335" s="886" t="n"/>
       <c r="AE335" s="886" t="n"/>
       <c r="AF335" s="886" t="n"/>
@@ -31558,29 +31558,29 @@
       <c r="D336" s="783" t="n"/>
       <c r="E336" s="778" t="n"/>
       <c r="F336" s="778" t="n"/>
-      <c r="G336" s="881" t="n"/>
-      <c r="H336" s="881" t="n"/>
-      <c r="I336" s="880" t="n"/>
-      <c r="J336" s="778" t="n"/>
-      <c r="K336" s="880" t="n"/>
+      <c r="G336" s="880" t="n"/>
+      <c r="H336" s="880" t="n"/>
+      <c r="I336" s="881" t="n"/>
+      <c r="J336" s="881" t="n"/>
+      <c r="K336" s="881" t="n"/>
       <c r="L336" s="778" t="n"/>
       <c r="M336" s="778" t="n"/>
-      <c r="N336" s="881" t="n"/>
-      <c r="O336" s="881" t="n"/>
+      <c r="N336" s="880" t="n"/>
+      <c r="O336" s="880" t="n"/>
       <c r="P336" s="778" t="n"/>
       <c r="Q336" s="778" t="n"/>
       <c r="R336" s="778" t="n"/>
       <c r="S336" s="778" t="n"/>
       <c r="T336" s="778" t="n"/>
-      <c r="U336" s="881" t="n"/>
-      <c r="V336" s="881" t="n"/>
+      <c r="U336" s="880" t="n"/>
+      <c r="V336" s="880" t="n"/>
       <c r="W336" s="778" t="n"/>
       <c r="X336" s="778" t="n"/>
       <c r="Y336" s="778" t="n"/>
       <c r="Z336" s="887" t="n"/>
       <c r="AA336" s="887" t="n"/>
-      <c r="AB336" s="880" t="n"/>
-      <c r="AC336" s="881" t="n"/>
+      <c r="AB336" s="881" t="n"/>
+      <c r="AC336" s="880" t="n"/>
       <c r="AD336" s="887" t="n"/>
       <c r="AE336" s="887" t="n"/>
       <c r="AF336" s="887" t="n"/>
@@ -31599,29 +31599,29 @@
       <c r="D337" s="755" t="n"/>
       <c r="E337" s="756" t="n"/>
       <c r="F337" s="756" t="n"/>
-      <c r="G337" s="879" t="n"/>
-      <c r="H337" s="879" t="n"/>
-      <c r="I337" s="878" t="n"/>
-      <c r="J337" s="756" t="n"/>
-      <c r="K337" s="878" t="n"/>
+      <c r="G337" s="878" t="n"/>
+      <c r="H337" s="878" t="n"/>
+      <c r="I337" s="879" t="n"/>
+      <c r="J337" s="879" t="n"/>
+      <c r="K337" s="879" t="n"/>
       <c r="L337" s="756" t="n"/>
       <c r="M337" s="756" t="n"/>
-      <c r="N337" s="879" t="n"/>
-      <c r="O337" s="879" t="n"/>
+      <c r="N337" s="878" t="n"/>
+      <c r="O337" s="878" t="n"/>
       <c r="P337" s="756" t="n"/>
       <c r="Q337" s="756" t="n"/>
       <c r="R337" s="756" t="n"/>
       <c r="S337" s="756" t="n"/>
       <c r="T337" s="756" t="n"/>
-      <c r="U337" s="879" t="n"/>
-      <c r="V337" s="879" t="n"/>
+      <c r="U337" s="878" t="n"/>
+      <c r="V337" s="878" t="n"/>
       <c r="W337" s="756" t="n"/>
       <c r="X337" s="756" t="n"/>
       <c r="Y337" s="756" t="n"/>
       <c r="Z337" s="886" t="n"/>
       <c r="AA337" s="886" t="n"/>
-      <c r="AB337" s="878" t="n"/>
-      <c r="AC337" s="879" t="n"/>
+      <c r="AB337" s="879" t="n"/>
+      <c r="AC337" s="878" t="n"/>
       <c r="AD337" s="886" t="n"/>
       <c r="AE337" s="886" t="n"/>
       <c r="AF337" s="886" t="n"/>
@@ -31640,29 +31640,29 @@
       <c r="D338" s="756" t="n"/>
       <c r="E338" s="756" t="n"/>
       <c r="F338" s="756" t="n"/>
-      <c r="G338" s="879" t="n"/>
-      <c r="H338" s="879" t="n"/>
-      <c r="I338" s="878" t="n"/>
-      <c r="J338" s="756" t="n"/>
-      <c r="K338" s="878" t="n"/>
+      <c r="G338" s="878" t="n"/>
+      <c r="H338" s="878" t="n"/>
+      <c r="I338" s="879" t="n"/>
+      <c r="J338" s="879" t="n"/>
+      <c r="K338" s="879" t="n"/>
       <c r="L338" s="756" t="n"/>
       <c r="M338" s="756" t="n"/>
-      <c r="N338" s="879" t="n"/>
-      <c r="O338" s="879" t="n"/>
+      <c r="N338" s="878" t="n"/>
+      <c r="O338" s="878" t="n"/>
       <c r="P338" s="756" t="n"/>
       <c r="Q338" s="756" t="n"/>
       <c r="R338" s="756" t="n"/>
       <c r="S338" s="756" t="n"/>
       <c r="T338" s="756" t="n"/>
-      <c r="U338" s="879" t="n"/>
-      <c r="V338" s="879" t="n"/>
+      <c r="U338" s="878" t="n"/>
+      <c r="V338" s="878" t="n"/>
       <c r="W338" s="756" t="n"/>
       <c r="X338" s="756" t="n"/>
       <c r="Y338" s="756" t="n"/>
       <c r="Z338" s="886" t="n"/>
       <c r="AA338" s="886" t="n"/>
-      <c r="AB338" s="878" t="n"/>
-      <c r="AC338" s="879" t="n"/>
+      <c r="AB338" s="879" t="n"/>
+      <c r="AC338" s="878" t="n"/>
       <c r="AD338" s="886" t="n"/>
       <c r="AE338" s="886" t="n"/>
       <c r="AF338" s="886" t="n"/>
@@ -31680,29 +31680,29 @@
       <c r="D339" s="783" t="n"/>
       <c r="E339" s="778" t="n"/>
       <c r="F339" s="778" t="n"/>
-      <c r="G339" s="881" t="n"/>
-      <c r="H339" s="881" t="n"/>
-      <c r="I339" s="880" t="n"/>
-      <c r="J339" s="778" t="n"/>
-      <c r="K339" s="880" t="n"/>
+      <c r="G339" s="880" t="n"/>
+      <c r="H339" s="880" t="n"/>
+      <c r="I339" s="881" t="n"/>
+      <c r="J339" s="881" t="n"/>
+      <c r="K339" s="881" t="n"/>
       <c r="L339" s="778" t="n"/>
       <c r="M339" s="778" t="n"/>
-      <c r="N339" s="881" t="n"/>
-      <c r="O339" s="881" t="n"/>
+      <c r="N339" s="880" t="n"/>
+      <c r="O339" s="880" t="n"/>
       <c r="P339" s="778" t="n"/>
       <c r="Q339" s="778" t="n"/>
       <c r="R339" s="778" t="n"/>
       <c r="S339" s="778" t="n"/>
       <c r="T339" s="778" t="n"/>
-      <c r="U339" s="881" t="n"/>
-      <c r="V339" s="881" t="n"/>
+      <c r="U339" s="880" t="n"/>
+      <c r="V339" s="880" t="n"/>
       <c r="W339" s="778" t="n"/>
       <c r="X339" s="778" t="n"/>
       <c r="Y339" s="778" t="n"/>
       <c r="Z339" s="887" t="n"/>
       <c r="AA339" s="887" t="n"/>
-      <c r="AB339" s="880" t="n"/>
-      <c r="AC339" s="881" t="n"/>
+      <c r="AB339" s="881" t="n"/>
+      <c r="AC339" s="880" t="n"/>
       <c r="AD339" s="887" t="n"/>
       <c r="AE339" s="887" t="n"/>
       <c r="AF339" s="887" t="n"/>
@@ -31720,29 +31720,29 @@
       <c r="D340" s="755" t="n"/>
       <c r="E340" s="755" t="n"/>
       <c r="F340" s="756" t="n"/>
-      <c r="G340" s="883" t="n"/>
-      <c r="H340" s="879" t="n"/>
-      <c r="I340" s="882" t="n"/>
-      <c r="J340" s="756" t="n"/>
-      <c r="K340" s="882" t="n"/>
+      <c r="G340" s="882" t="n"/>
+      <c r="H340" s="878" t="n"/>
+      <c r="I340" s="883" t="n"/>
+      <c r="J340" s="879" t="n"/>
+      <c r="K340" s="883" t="n"/>
       <c r="L340" s="756" t="n"/>
       <c r="M340" s="756" t="n"/>
-      <c r="N340" s="883" t="n"/>
-      <c r="O340" s="883" t="n"/>
+      <c r="N340" s="882" t="n"/>
+      <c r="O340" s="882" t="n"/>
       <c r="P340" s="756" t="n"/>
       <c r="Q340" s="756" t="n"/>
       <c r="R340" s="755" t="n"/>
       <c r="S340" s="756" t="n"/>
       <c r="T340" s="756" t="n"/>
-      <c r="U340" s="883" t="n"/>
-      <c r="V340" s="883" t="n"/>
+      <c r="U340" s="882" t="n"/>
+      <c r="V340" s="882" t="n"/>
       <c r="W340" s="756" t="n"/>
       <c r="X340" s="756" t="n"/>
       <c r="Y340" s="755" t="n"/>
       <c r="Z340" s="886" t="n"/>
       <c r="AA340" s="886" t="n"/>
-      <c r="AB340" s="882" t="n"/>
-      <c r="AC340" s="883" t="n"/>
+      <c r="AB340" s="883" t="n"/>
+      <c r="AC340" s="882" t="n"/>
       <c r="AD340" s="886" t="n"/>
       <c r="AE340" s="886" t="n"/>
       <c r="AF340" s="888" t="n"/>
@@ -31760,29 +31760,29 @@
       <c r="D341" s="756" t="n"/>
       <c r="E341" s="756" t="n"/>
       <c r="F341" s="756" t="n"/>
-      <c r="G341" s="879" t="n"/>
-      <c r="H341" s="879" t="n"/>
-      <c r="I341" s="878" t="n"/>
-      <c r="J341" s="756" t="n"/>
-      <c r="K341" s="878" t="n"/>
+      <c r="G341" s="878" t="n"/>
+      <c r="H341" s="878" t="n"/>
+      <c r="I341" s="879" t="n"/>
+      <c r="J341" s="879" t="n"/>
+      <c r="K341" s="879" t="n"/>
       <c r="L341" s="756" t="n"/>
       <c r="M341" s="756" t="n"/>
-      <c r="N341" s="879" t="n"/>
-      <c r="O341" s="879" t="n"/>
+      <c r="N341" s="878" t="n"/>
+      <c r="O341" s="878" t="n"/>
       <c r="P341" s="756" t="n"/>
       <c r="Q341" s="756" t="n"/>
       <c r="R341" s="756" t="n"/>
       <c r="S341" s="756" t="n"/>
       <c r="T341" s="756" t="n"/>
-      <c r="U341" s="879" t="n"/>
-      <c r="V341" s="879" t="n"/>
+      <c r="U341" s="878" t="n"/>
+      <c r="V341" s="878" t="n"/>
       <c r="W341" s="756" t="n"/>
       <c r="X341" s="756" t="n"/>
       <c r="Y341" s="756" t="n"/>
       <c r="Z341" s="886" t="n"/>
       <c r="AA341" s="886" t="n"/>
-      <c r="AB341" s="878" t="n"/>
-      <c r="AC341" s="879" t="n"/>
+      <c r="AB341" s="879" t="n"/>
+      <c r="AC341" s="878" t="n"/>
       <c r="AD341" s="886" t="n"/>
       <c r="AE341" s="886" t="n"/>
       <c r="AF341" s="886" t="n"/>
@@ -31800,29 +31800,29 @@
       <c r="D342" s="756" t="n"/>
       <c r="E342" s="756" t="n"/>
       <c r="F342" s="756" t="n"/>
-      <c r="G342" s="879" t="n"/>
-      <c r="H342" s="879" t="n"/>
-      <c r="I342" s="878" t="n"/>
-      <c r="J342" s="756" t="n"/>
-      <c r="K342" s="878" t="n"/>
+      <c r="G342" s="878" t="n"/>
+      <c r="H342" s="878" t="n"/>
+      <c r="I342" s="879" t="n"/>
+      <c r="J342" s="879" t="n"/>
+      <c r="K342" s="879" t="n"/>
       <c r="L342" s="756" t="n"/>
       <c r="M342" s="756" t="n"/>
-      <c r="N342" s="879" t="n"/>
-      <c r="O342" s="879" t="n"/>
+      <c r="N342" s="878" t="n"/>
+      <c r="O342" s="878" t="n"/>
       <c r="P342" s="756" t="n"/>
       <c r="Q342" s="756" t="n"/>
       <c r="R342" s="756" t="n"/>
       <c r="S342" s="756" t="n"/>
       <c r="T342" s="756" t="n"/>
-      <c r="U342" s="879" t="n"/>
-      <c r="V342" s="879" t="n"/>
+      <c r="U342" s="878" t="n"/>
+      <c r="V342" s="878" t="n"/>
       <c r="W342" s="756" t="n"/>
       <c r="X342" s="756" t="n"/>
       <c r="Y342" s="756" t="n"/>
       <c r="Z342" s="886" t="n"/>
       <c r="AA342" s="886" t="n"/>
-      <c r="AB342" s="878" t="n"/>
-      <c r="AC342" s="879" t="n"/>
+      <c r="AB342" s="879" t="n"/>
+      <c r="AC342" s="878" t="n"/>
       <c r="AD342" s="886" t="n"/>
       <c r="AE342" s="886" t="n"/>
       <c r="AF342" s="886" t="n"/>

</xml_diff>

<commit_message>
Usa el calendari laboral 2027 corregit (graella acolorida i dies laborables per mes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDkSHuGdwYQW6bQEdBsCTx
</commit_message>
<xml_diff>
--- a/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
+++ b/cronograma/CRONOGRAMA_26-27_PROVISIONAL.xlsx
@@ -29398,7 +29398,7 @@
       <c r="AG265" s="156" t="n"/>
       <c r="AH265" s="142" t="n"/>
       <c r="AI265" s="500" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="266" ht="51" customHeight="1" s="757">
@@ -32021,11 +32021,11 @@
       <c r="AG332" s="156" t="n"/>
       <c r="AH332" s="142" t="n"/>
       <c r="AI332" s="500" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AK332" s="898" t="inlineStr">
         <is>
-          <t>Festius: 06/12 Dia de la Constitució (Nacional) · 07/12 Festiu local (canvi pel 15/09) · 08/12 Immaculada Concepció (Nacional) · 25/12 Nadal (Nacional) · Vacances: 23/12–31/12</t>
+          <t>Festius: 06/12 Dia de la Constitució (Nacional) · 07/12 Festiu Multimèdia · 08/12 Immaculada Concepció (Nacional) · 25/12 Nadal (Nacional) · Vacances: 24/12–31/12</t>
         </is>
       </c>
     </row>
@@ -32170,7 +32170,7 @@
       <c r="W334" s="756" t="n"/>
       <c r="X334" s="756" t="n"/>
       <c r="Y334" s="756" t="n"/>
-      <c r="Z334" s="907" t="n"/>
+      <c r="Z334" s="756" t="n"/>
       <c r="AA334" s="907" t="n"/>
       <c r="AB334" s="900" t="n"/>
       <c r="AC334" s="899" t="n"/>
@@ -32211,7 +32211,7 @@
       <c r="W335" s="756" t="n"/>
       <c r="X335" s="756" t="n"/>
       <c r="Y335" s="756" t="n"/>
-      <c r="Z335" s="907" t="n"/>
+      <c r="Z335" s="756" t="n"/>
       <c r="AA335" s="907" t="n"/>
       <c r="AB335" s="900" t="n"/>
       <c r="AC335" s="899" t="n"/>
@@ -32252,7 +32252,7 @@
       <c r="W336" s="778" t="n"/>
       <c r="X336" s="778" t="n"/>
       <c r="Y336" s="778" t="n"/>
-      <c r="Z336" s="908" t="n"/>
+      <c r="Z336" s="778" t="n"/>
       <c r="AA336" s="908" t="n"/>
       <c r="AB336" s="902" t="n"/>
       <c r="AC336" s="901" t="n"/>
@@ -32293,7 +32293,7 @@
       <c r="W337" s="756" t="n"/>
       <c r="X337" s="756" t="n"/>
       <c r="Y337" s="756" t="n"/>
-      <c r="Z337" s="907" t="n"/>
+      <c r="Z337" s="756" t="n"/>
       <c r="AA337" s="907" t="n"/>
       <c r="AB337" s="900" t="n"/>
       <c r="AC337" s="899" t="n"/>
@@ -32334,7 +32334,7 @@
       <c r="W338" s="756" t="n"/>
       <c r="X338" s="756" t="n"/>
       <c r="Y338" s="756" t="n"/>
-      <c r="Z338" s="907" t="n"/>
+      <c r="Z338" s="756" t="n"/>
       <c r="AA338" s="907" t="n"/>
       <c r="AB338" s="900" t="n"/>
       <c r="AC338" s="899" t="n"/>
@@ -32374,7 +32374,7 @@
       <c r="W339" s="778" t="n"/>
       <c r="X339" s="778" t="n"/>
       <c r="Y339" s="778" t="n"/>
-      <c r="Z339" s="908" t="n"/>
+      <c r="Z339" s="778" t="n"/>
       <c r="AA339" s="908" t="n"/>
       <c r="AB339" s="902" t="n"/>
       <c r="AC339" s="901" t="n"/>
@@ -32414,7 +32414,7 @@
       <c r="W340" s="756" t="n"/>
       <c r="X340" s="756" t="n"/>
       <c r="Y340" s="755" t="n"/>
-      <c r="Z340" s="907" t="n"/>
+      <c r="Z340" s="756" t="n"/>
       <c r="AA340" s="907" t="n"/>
       <c r="AB340" s="904" t="n"/>
       <c r="AC340" s="903" t="n"/>
@@ -32454,7 +32454,7 @@
       <c r="W341" s="756" t="n"/>
       <c r="X341" s="756" t="n"/>
       <c r="Y341" s="756" t="n"/>
-      <c r="Z341" s="907" t="n"/>
+      <c r="Z341" s="756" t="n"/>
       <c r="AA341" s="907" t="n"/>
       <c r="AB341" s="900" t="n"/>
       <c r="AC341" s="899" t="n"/>
@@ -32494,7 +32494,7 @@
       <c r="W342" s="756" t="n"/>
       <c r="X342" s="756" t="n"/>
       <c r="Y342" s="756" t="n"/>
-      <c r="Z342" s="907" t="n"/>
+      <c r="Z342" s="756" t="n"/>
       <c r="AA342" s="907" t="n"/>
       <c r="AB342" s="900" t="n"/>
       <c r="AC342" s="899" t="n"/>
@@ -34515,7 +34515,7 @@
     <row r="43">
       <c r="A43" s="941" t="inlineStr">
         <is>
-          <t>• Setembre-desembre 2027: festius i vacances del CALENDARI_LABORAL_2027 (els festius locals 04/09 i 15/09 hi consten com 'a omplir'). S'hi afegeix el 12/10 com a festiu.</t>
+          <t>• 2027: festius, vacances i dies laborables segons la graella 'Calendari 2027' del CALENDARI_LABORAL_2027 corregit (12/10 festiu; 04/09 i 15/09 laborables a canvi del 25/06 i 07/12, festius Multimèdia; vacances de Nadal 24-31/12).</t>
         </is>
       </c>
     </row>

</xml_diff>